<commit_message>
fix(baba): correct 2025-06-30 6-K source_url (was AGM circular, now Q1 FY26 earnings)
The DB row for BABA form_type=6-K period_of_report=2025-06-30 had
source_url pointing at accession 0001104659-25-074564 — which is
Alibaba's annual-meeting shareholder circular (filed 2025-08-06),
NOT the Q1 FY26 earnings announcement. That's why the original
BABA-6K regex found no Cloud Intelligence Group line there.

The real Q1 FY26 earnings 6-K was filed 2025-08-29 under accession
0001104659-25-085638 (file tm2524743d1_ex99-1.htm, 473KB). It
reports "revenue from Cloud Intelligence Group was RMB33,398
million" for the quarter ended June 30, 2025.

Updated source_url in place, re-ran scripts/extract_baba_cloud_6k.py
and reconcile. BABA calendar 2025Q2 now = $4.66B on the chart, and
the year is internally consistent with the 20-F annual.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workbook/capex_tracker.xlsx
+++ b/workbook/capex_tracker.xlsx
@@ -2041,7 +2041,7 @@
         <t>Source: [BABA] FY2025 6-K (filed 2025-08-06)
 Derivation:
   Derived: 9M = Q1+Q2+Q3
-Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925074564/tm2522605d1_ex99-2.htm</t>
+Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925085638/tm2524743d1_ex99-1.htm</t>
       </text>
     </comment>
     <comment ref="AR5" authorId="0" shapeId="0">
@@ -9666,6 +9666,17 @@
 Report: https://www.sec.gov/Archives/edgar/data/1577552/000095017025090161/baba-20250331.htm</t>
       </text>
     </comment>
+    <comment ref="AQ5" authorId="0" shapeId="0">
+      <text>
+        <t>Source: [BABA] FY2025 6-K (filed 2025-08-06)
+Section: 6-K Press Release — Cloud Intelligence Group
+Line item: "Cloud Intelligence Group For the quarter ended June 30, 2025, revenue from Cloud Intelligence Group was RMB33,398 million"
+Value: CNY 33,398M → $4,661M USD
+FX: CNY/USD 0.1396 @ 2025-06-30 (source: ECB via frankfurter.app)
+Method: baba-cloud-6k@0.1.0
+Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925085638/tm2524743d1_ex99-1.htm</t>
+      </text>
+    </comment>
     <comment ref="AR5" authorId="0" shapeId="0">
       <text>
         <t>Source: [BABA] FY2025 6-K (filed 2025-11-25)
@@ -19648,7 +19659,7 @@
         <t>Source: [BABA] FY2025 6-K (filed 2025-08-06)
 Derivation:
   Derived: 9M = Q1+Q2+Q3
-Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925074564/tm2522605d1_ex99-2.htm</t>
+Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925085638/tm2524743d1_ex99-1.htm</t>
       </text>
     </comment>
     <comment ref="AS20" authorId="0" shapeId="0">
@@ -20071,6 +20082,17 @@
 FX: CNY/USD 0.1379 @ 2025-03-31 (source: ECB via frankfurter.app)
 Method: claude-code
 Report: https://www.sec.gov/Archives/edgar/data/1577552/000095017025090161/baba-20250331.htm</t>
+      </text>
+    </comment>
+    <comment ref="AR21" authorId="0" shapeId="0">
+      <text>
+        <t>Source: [BABA] FY2025 6-K (filed 2025-08-06)
+Section: 6-K Press Release — Cloud Intelligence Group
+Line item: "Cloud Intelligence Group For the quarter ended June 30, 2025, revenue from Cloud Intelligence Group was RMB33,398 million"
+Value: CNY 33,398M → $4,661M USD
+FX: CNY/USD 0.1396 @ 2025-06-30 (source: ECB via frankfurter.app)
+Method: baba-cloud-6k@0.1.0
+Report: https://www.sec.gov/Archives/edgar/data/1577552/000110465925085638/tm2524743d1_ex99-1.htm</t>
       </text>
     </comment>
     <comment ref="AS21" authorId="0" shapeId="0">
@@ -29593,7 +29615,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-04-18 21:47 UTC</t>
+          <t>2026-04-19 15:09 UTC</t>
         </is>
       </c>
     </row>
@@ -29617,7 +29639,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2560</t>
+          <t>2561</t>
         </is>
       </c>
     </row>
@@ -30109,7 +30131,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-18 21:47 UTC</t>
+          <t>2026-04-19 15:09 UTC</t>
         </is>
       </c>
     </row>
@@ -30120,7 +30142,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2560</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="5">
@@ -30284,7 +30306,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -36228,6 +36250,9 @@
       </c>
       <c r="AP5" s="9" t="n">
         <v>16273</v>
+      </c>
+      <c r="AQ5" s="9" t="n">
+        <v>4661</v>
       </c>
       <c r="AR5" s="9" t="n">
         <v>5594</v>
@@ -41067,6 +41092,9 @@
       <c r="AQ21" s="9" t="n">
         <v>16273</v>
       </c>
+      <c r="AR21" s="9" t="n">
+        <v>4661</v>
+      </c>
       <c r="AS21" s="9" t="n">
         <v>5594</v>
       </c>

</xml_diff>